<commit_message>
Schedule 12–25.10: wording after review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015DfynR8ViCbDyQMuNVS5SH
</commit_message>
<xml_diff>
--- a/content/plan/raspisanie-12-25.10.xlsx
+++ b/content/plan/raspisanie-12-25.10.xlsx
@@ -721,7 +721,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Рилс «Знакомьтесь, это зубр» (12:00) + карусель 5 сл. (18:00) · CTA: подпишитесь</t>
+          <t>Рилс «Знакомьтесь, это зубр» (12:00, версия без звука + трендовый трек, удар на 2-й секунде) + карусель 5 сл. (18:00) · CTA: подпишитесь</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Сколько стоит потерянный клиент</t>
+          <t>Сколько стоит потерянный клиент + чек-лист «12 причин» (PDF)</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>5 фраз, которые удерживают после пробного</t>
+          <t>5 фраз, которые удерживают клиента после пробного занятия</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -1055,12 +1055,12 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Мем + рилс · голосование</t>
+          <t>Мем + рилс</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>«Нет / Да» про форумы + рилс «Полный зал»</t>
+          <t>«Нет / Да» про форумы (верх — ч/б зубр) + рилс «Полный зал»</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">

</xml_diff>